<commit_message>
aggiustati parametri coorte con caratterizzazione
</commit_message>
<xml_diff>
--- a/p_parameters/archive_parameters/codebooks/D3_coorte_con_caratterizzazione.xlsx
+++ b/p_parameters/archive_parameters/codebooks/D3_coorte_con_caratterizzazione.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
   <si>
     <t xml:space="preserve">parameter</t>
   </si>
@@ -64,30 +64,6 @@
     <t xml:space="preserve">Bypass</t>
   </si>
   <si>
-    <t xml:space="preserve">anticol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">antipsico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sulfo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ins_rapida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ins_lunga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ppi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anticoag</t>
-  </si>
-  <si>
     <t xml:space="preserve">ese_cardio</t>
   </si>
   <si>
@@ -134,30 +110,6 @@
   </si>
   <si>
     <t xml:space="preserve">ese_altra_cronica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_anticol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_fans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_antipsico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_sulfo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_ins_rapida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_ins_lunga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_ppi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">med_anticoag</t>
   </si>
 </sst>
 </file>
@@ -417,155 +369,205 @@
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="0"/>
-      <c r="D2" s="0"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>6</v>
+      <c r="A6" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
+      <c r="D6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>-99999</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
+      <c r="D7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
+      <c r="D8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="0"/>
-      <c r="D9" s="0"/>
+      <c r="D9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="0"/>
-      <c r="D10" s="0"/>
+      <c r="D10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="0"/>
-      <c r="D11" s="0"/>
+      <c r="D11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="0"/>
-      <c r="D12" s="0"/>
+      <c r="D12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="0" t="s">
+      <c r="A13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="0"/>
-      <c r="D13" s="0"/>
+      <c r="D13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>-365</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="0"/>
-      <c r="D14" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="0" t="n">
-        <v>-99999</v>
-      </c>
-      <c r="F14" s="0" t="n">
+      <c r="D14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>-1094</v>
+      </c>
+      <c r="F14" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
@@ -576,14 +578,13 @@
       <c r="B15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="0"/>
-      <c r="D15" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="0" t="n">
+      <c r="D15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="1" t="n">
         <v>-1094</v>
       </c>
-      <c r="F15" s="0" t="n">
+      <c r="F15" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
@@ -594,429 +595,222 @@
       <c r="B16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="0"/>
-      <c r="D16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="0" t="n">
+      <c r="D16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="1" t="n">
         <v>-1094</v>
       </c>
-      <c r="F16" s="0" t="n">
+      <c r="F16" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="0"/>
-      <c r="D17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F17" s="0" t="n">
+      <c r="D17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>-99999</v>
+      </c>
+      <c r="F17" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="0"/>
-      <c r="D18" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="0" t="n">
+      <c r="D18" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1" t="n">
         <v>-1094</v>
       </c>
-      <c r="F18" s="0" t="n">
+      <c r="F18" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="0"/>
-      <c r="D19" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F19" s="0" t="n">
+      <c r="D19" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>-99999</v>
+      </c>
+      <c r="F19" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="0"/>
-      <c r="D20" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="0" t="n">
+      <c r="D20" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="1" t="n">
         <v>-1094</v>
       </c>
-      <c r="F20" s="0" t="n">
+      <c r="F20" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="0"/>
-      <c r="D21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F21" s="0" t="n">
+      <c r="D21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>-99999</v>
+      </c>
+      <c r="F21" s="1" t="n">
         <v>-365</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="0"/>
-      <c r="D22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F22" s="0" t="n">
-        <v>-365</v>
-      </c>
+      <c r="A22" s="5"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="0"/>
-      <c r="D23" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F23" s="0" t="n">
-        <v>-365</v>
-      </c>
+      <c r="A23" s="5"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="0"/>
-      <c r="D24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F24" s="0" t="n">
-        <v>-365</v>
-      </c>
+      <c r="A24" s="5"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="0"/>
-      <c r="D25" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="0" t="n">
-        <v>-99999</v>
-      </c>
-      <c r="F25" s="0" t="n">
-        <v>-365</v>
-      </c>
+      <c r="A25" s="5"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="0"/>
-      <c r="D26" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F26" s="0" t="n">
-        <v>-365</v>
-      </c>
+      <c r="A26" s="5"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="0"/>
-      <c r="D27" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="0" t="n">
-        <v>-99999</v>
-      </c>
-      <c r="F27" s="0" t="n">
-        <v>-365</v>
-      </c>
+      <c r="A27" s="5"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C28" s="0"/>
-      <c r="D28" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="0" t="n">
-        <v>-1094</v>
-      </c>
-      <c r="F28" s="0" t="n">
-        <v>-365</v>
-      </c>
+      <c r="A28" s="5"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" s="0"/>
-      <c r="D29" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="0" t="n">
-        <v>-99999</v>
-      </c>
-      <c r="F29" s="0" t="n">
-        <v>-365</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30" s="0"/>
-      <c r="D30" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F30" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C31" s="0"/>
-      <c r="D31" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F31" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="A31" s="5"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C32" s="0"/>
-      <c r="D32" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F32" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="A32" s="5"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C33" s="0"/>
-      <c r="D33" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F33" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="1"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="0"/>
-      <c r="D34" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F34" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="1"/>
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C35" s="0"/>
-      <c r="D35" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F35" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="A35" s="5"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
       <c r="G35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C36" s="0"/>
-      <c r="D36" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="E36" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F36" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="1"/>
+      <c r="A36" s="5"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C37" s="0"/>
-      <c r="D37" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="0" t="n">
-        <v>-365</v>
-      </c>
-      <c r="F37" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="A37" s="7"/>
+      <c r="B37" s="8"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0"/>
-      <c r="C38" s="0"/>
-      <c r="D38" s="0"/>
+      <c r="A38" s="7"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5"/>
+      <c r="A39" s="7"/>
       <c r="D39" s="6"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5"/>
+      <c r="A40" s="7"/>
+      <c r="B40" s="9"/>
       <c r="D40" s="6"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
+      <c r="A41" s="7"/>
+      <c r="B41" s="9"/>
       <c r="D41" s="6"/>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
       <c r="D42" s="6"/>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -1026,7 +820,6 @@
       <c r="D43" s="6"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5"/>
@@ -1035,131 +828,87 @@
       <c r="F44" s="1"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7"/>
-      <c r="B45" s="8"/>
+      <c r="A45" s="5"/>
       <c r="D45" s="6"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7"/>
+      <c r="A46" s="5"/>
       <c r="D46" s="6"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7"/>
+      <c r="A47" s="5"/>
       <c r="D47" s="6"/>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7"/>
-      <c r="B48" s="9"/>
-      <c r="D48" s="6"/>
+      <c r="A48" s="5"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7"/>
-      <c r="B49" s="9"/>
-      <c r="D49" s="6"/>
+      <c r="A49" s="5"/>
+      <c r="B49" s="6"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5"/>
-      <c r="D50" s="6"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5"/>
-      <c r="D51" s="6"/>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5"/>
-      <c r="D52" s="6"/>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5"/>
-      <c r="D53" s="6"/>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5"/>
-      <c r="D54" s="6"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5"/>
-      <c r="D55" s="6"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="5"/>
+      <c r="A56" s="10"/>
+      <c r="B56" s="10"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
     </row>
-    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="5"/>
-      <c r="B57" s="6"/>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-    </row>
-    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5"/>
-      <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-    </row>
-    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="5"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-    </row>
-    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5"/>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-    </row>
-    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="5"/>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-    </row>
-    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5"/>
-      <c r="E62" s="1"/>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-    </row>
-    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="5"/>
-      <c r="E63" s="1"/>
-      <c r="F63" s="1"/>
-      <c r="G63" s="1"/>
-    </row>
-    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="10"/>
-      <c r="B64" s="10"/>
-      <c r="E64" s="1"/>
-      <c r="F64" s="1"/>
-      <c r="G64" s="1"/>
-    </row>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>